<commit_message>
Legacy content cleanup — regenerated templates, aligned docs/downloads with templates/
- Regenerated all xlsx templates from cleaned csv sources
- Re-stamped manifest.json with the current vocabulary (action/memory/flow)
- Fixed scripts/create_templates.py source of scope-document.xlsx legacy content
- Propagated clean binaries to docs/downloads/ (previously even more stale than templates/)
- Replaced 'Core banking vendor' example in personalise/prompts/learning/csm-discovery.md
- .github/workflows/deploy.yml: Node.js 24 opt-in to remove deprecation warnings
</commit_message>
<xml_diff>
--- a/docs/downloads/Stage 1 - Decompose.xlsx
+++ b/docs/downloads/Stage 1 - Decompose.xlsx
@@ -1325,7 +1325,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Yes — automating the health review would produce structured JSON output (typed scores, risk objects with severity/evidence fields, trend data with direction and magnitude). The EBR prep workflow could consume this directly via the state schema instead of the CSM re-reading their own prose report.</t>
+          <t>Yes — automating the health review would produce structured JSON output (typed scores, risk objects with severity/evidence fields, trend data with direction and magnitude). The EBR prep workflow could consume this directly via the memory schema instead of the CSM re-reading their own prose report.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Partial — automating the health review builds the Mixpanel data-retrieval and usage-analysis tools. The upsell workflow needs the same raw data but applies different analysis logic (threshold comparison vs. scoring), so the retrieval tools transfer but the analysis nodes do not.</t>
+          <t>Partial — automating the health review builds the Mixpanel data-retrieval and usage-analysis tools. The upsell workflow needs the same raw data but applies different analysis logic (threshold comparison vs. scoring), so the retrieval tools transfer but the analysis actions do not.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>The Mixpanel connector and usage data transformation are reusable. The analysis logic is workflow-specific — health scoring vs. expansion signal detection require different prompts and different output schemas. Plan to reuse the data layer but expect to build new analysis nodes.</t>
+          <t>The Mixpanel connector and usage data transformation are reusable. The analysis logic is workflow-specific — health scoring vs. expansion signal detection require different prompts and different output schemas. Plan to reuse the data layer but expect to build new analysis actions.</t>
         </is>
       </c>
     </row>

</xml_diff>